<commit_message>
Etappe 2: Mail-Parser, kicker-Import, Echtlauf 2. Spieltag
</commit_message>
<xml_diff>
--- a/daten/spielerbasis/Spielerbasis_2026-27.xlsx
+++ b/daten/spielerbasis/Spielerbasis_2026-27.xlsx
@@ -5061,6 +5061,11 @@
           <t>exakt</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>kicker schreibt im Schema 'Kai. Sano'</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">

</xml_diff>